<commit_message>
Implementación RAY y benchmarks actualizados + Docker tar
</commit_message>
<xml_diff>
--- a/benchmark_cnn_hpc_metricas.xlsx
+++ b/benchmark_cnn_hpc_metricas.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andym\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andym\CLASES\SEMESTRE 9\COMPUTACION DE ALTO RENDIMIENTO\CNN-optimization-with-HPC-tools-\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F39FA1A4-C90E-4B0A-A4ED-1A041E203122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -16,41 +16,6 @@
     <sheet name="Benchmark CNN HPC" sheetId="1" r:id="rId1"/>
     <sheet name="Instrucciones" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'Benchmark CNN HPC'!$A$2:$B$13</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'Benchmark CNN HPC'!$C$1</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">'Benchmark CNN HPC'!$G$2:$G$13</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">'Benchmark CNN HPC'!$H$1</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">'Benchmark CNN HPC'!$H$2:$H$13</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">'Benchmark CNN HPC'!$I$1</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">'Benchmark CNN HPC'!$I$2:$I$13</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">'Benchmark CNN HPC'!$J$1</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">'Benchmark CNN HPC'!$J$2:$J$13</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">'Benchmark CNN HPC'!$K$1</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">'Benchmark CNN HPC'!$K$2:$K$13</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">'Benchmark CNN HPC'!$L$1</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'Benchmark CNN HPC'!$C$2:$C$13</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">'Benchmark CNN HPC'!$L$2:$L$13</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">'Benchmark CNN HPC'!$M$1</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">'Benchmark CNN HPC'!$M$2:$M$13</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">'Benchmark CNN HPC'!$N$1</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">'Benchmark CNN HPC'!$N$2:$N$13</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">'Benchmark CNN HPC'!$O$1</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">'Benchmark CNN HPC'!$O$2:$O$13</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">'Benchmark CNN HPC'!$P$1</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">'Benchmark CNN HPC'!$P$2:$P$13</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">'Benchmark CNN HPC'!$Q$1</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'Benchmark CNN HPC'!$D$1</definedName>
-    <definedName name="_xlchart.v1.30" hidden="1">'Benchmark CNN HPC'!$Q$2:$Q$13</definedName>
-    <definedName name="_xlchart.v1.31" hidden="1">'Benchmark CNN HPC'!$R$1</definedName>
-    <definedName name="_xlchart.v1.32" hidden="1">'Benchmark CNN HPC'!$R$2:$R$13</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'Benchmark CNN HPC'!$D$2:$D$13</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'Benchmark CNN HPC'!$E$1</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">'Benchmark CNN HPC'!$E$2:$E$13</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">'Benchmark CNN HPC'!$F$1</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">'Benchmark CNN HPC'!$F$2:$F$13</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">'Benchmark CNN HPC'!$G$1</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
@@ -275,17 +240,17 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>